<commit_message>
Padatkan timeline rencana kerja jadi 3 hari (Fase 1-5)
Fase 6 (finalisasi) dan Fase 7 (duplikasi) dipindah ke kolom
"Lanjutan" karena keduanya memang pekerjaan setelah unit pertama
terbukti jalan, bukan bagian dari uji coba awal.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Rencana-Kerja.xlsx
+++ b/Rencana-Kerja.xlsx
@@ -148,6 +148,10 @@
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -155,14 +159,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -627,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -756,85 +756,86 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>TARGET 3 HARI (Fase 1-5)</t>
+        </is>
+      </c>
+      <c r="B13" s="9">
+        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$F$5:$F$74,"D1")+SUMIFS(ToDo!$E$5:$E$74,ToDo!$F$5:$F$74,"D2")+SUMIFS(ToDo!$E$5:$E$74,ToDo!$F$5:$F$74,"D3")</f>
+        <v/>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>jam - rata-rata dibagi 3 hari</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Sisanya (Fase 6-7, Lanjutan)</t>
+        </is>
+      </c>
+      <c r="B14" s="6">
+        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$F$5:$F$74,"Lanjutan")</f>
+        <v/>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>jam - finalisasi &amp; duplikasi, di luar target 3 hari</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>Rincian per Fase</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>Tugas</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>Selesai</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>Progres</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>Jam</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F17" s="11" t="inlineStr">
         <is>
           <t>Jam Tersisa</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr">
+      <c r="G17" s="11" t="inlineStr">
         <is>
           <t>Gate</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>Fase 0 - Verifikasi Meja</t>
-        </is>
-      </c>
-      <c r="B17" s="4">
-        <f>COUNTIF(ToDo!$B$5:$B$74,$A17)</f>
-        <v/>
-      </c>
-      <c r="C17" s="4">
-        <f>COUNTIFS(ToDo!$B$5:$B$74,$A17,ToDo!$I$5:$I$74,"Selesai")</f>
-        <v/>
-      </c>
-      <c r="D17" s="5">
-        <f>IFERROR(C17/B17,0)</f>
-        <v/>
-      </c>
-      <c r="E17" s="6">
-        <f>SUMIF(ToDo!$B$5:$B$74,$A17,ToDo!$E$5:$E$74)</f>
-        <v/>
-      </c>
-      <c r="F17" s="6">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A17,ToDo!$I$5:$I$74,"Belum")</f>
-        <v/>
-      </c>
-      <c r="G17" s="4">
-        <f>COUNTIFS(ToDo!$B$5:$B$74,$A17,ToDo!$H$5:$H$74,"Ya")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>Fase 1 - Wiring &amp; Daya</t>
         </is>
       </c>
       <c r="B18" s="4">
@@ -863,9 +864,9 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>Fase 2 - Flash &amp; Bench</t>
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Fase 1 - Wiring &amp; Daya</t>
         </is>
       </c>
       <c r="B19" s="4">
@@ -894,9 +895,9 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>Fase 3 - Failsafe &amp; Integrasi</t>
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Fase 2 - Flash &amp; Bench</t>
         </is>
       </c>
       <c r="B20" s="4">
@@ -925,9 +926,9 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>Fase 4 - Uji Lantai &amp; Tuning</t>
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>Fase 3 - Failsafe &amp; Integrasi</t>
         </is>
       </c>
       <c r="B21" s="4">
@@ -956,9 +957,9 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>Fase 5 - Pindah ke LattePanda</t>
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>Fase 4 - Uji Lantai &amp; Tuning</t>
         </is>
       </c>
       <c r="B22" s="4">
@@ -987,9 +988,9 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>Fase 6 - Finalisasi</t>
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>Fase 5 - Pindah ke LattePanda</t>
         </is>
       </c>
       <c r="B23" s="4">
@@ -1018,9 +1019,9 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>Fase 7 - Duplikasi &amp; Produksi</t>
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Fase 6 - Finalisasi</t>
         </is>
       </c>
       <c r="B24" s="4">
@@ -1049,33 +1050,64 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Fase 7 - Duplikasi &amp; Produksi</t>
+        </is>
+      </c>
+      <c r="B25" s="4">
+        <f>COUNTIF(ToDo!$B$5:$B$74,$A25)</f>
+        <v/>
+      </c>
+      <c r="C25" s="4">
+        <f>COUNTIFS(ToDo!$B$5:$B$74,$A25,ToDo!$I$5:$I$74,"Selesai")</f>
+        <v/>
+      </c>
+      <c r="D25" s="5">
+        <f>IFERROR(C25/B25,0)</f>
+        <v/>
+      </c>
+      <c r="E25" s="6">
+        <f>SUMIF(ToDo!$B$5:$B$74,$A25,ToDo!$E$5:$E$74)</f>
+        <v/>
+      </c>
+      <c r="F25" s="6">
+        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A25,ToDo!$I$5:$I$74,"Belum")</f>
+        <v/>
+      </c>
+      <c r="G25" s="4">
+        <f>COUNTIFS(ToDo!$B$5:$B$74,$A25,ToDo!$H$5:$H$74,"Ya")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B25" s="12">
-        <f>SUM(B17:B24)</f>
-        <v/>
-      </c>
-      <c r="C25" s="12">
-        <f>SUM(C17:C24)</f>
-        <v/>
-      </c>
-      <c r="D25" s="13">
-        <f>IFERROR(C25/B25,0)</f>
-        <v/>
-      </c>
-      <c r="E25" s="14">
-        <f>SUM(E17:E24)</f>
-        <v/>
-      </c>
-      <c r="F25" s="14">
-        <f>SUM(F17:F24)</f>
-        <v/>
-      </c>
-      <c r="G25" s="12">
-        <f>SUM(G17:G24)</f>
+      <c r="B26" s="13">
+        <f>SUM(B18:B25)</f>
+        <v/>
+      </c>
+      <c r="C26" s="13">
+        <f>SUM(C18:C25)</f>
+        <v/>
+      </c>
+      <c r="D26" s="14">
+        <f>IFERROR(C26/B26,0)</f>
+        <v/>
+      </c>
+      <c r="E26" s="9">
+        <f>SUM(E18:E25)</f>
+        <v/>
+      </c>
+      <c r="F26" s="9">
+        <f>SUM(F18:F25)</f>
+        <v/>
+      </c>
+      <c r="G26" s="13">
+        <f>SUM(G18:G25)</f>
         <v/>
       </c>
     </row>
@@ -1120,52 +1152,52 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>Tugas</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>Kriteria Sukses / Catatan</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>Jam</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr">
         <is>
           <t>Hari</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>Prioritas</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="H4" s="11" t="inlineStr">
         <is>
           <t>Gate</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="J4" s="9" t="inlineStr">
+      <c r="J4" s="11" t="inlineStr">
         <is>
           <t>Referensi</t>
         </is>
@@ -1177,17 +1209,17 @@
           <t>0.1</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Fase 0 - Verifikasi Meja</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>Ground station Python + simulator</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>95 uji otomatis lulus (protokol, kurva, config, MJPEG)</t>
         </is>
@@ -1215,7 +1247,7 @@
           <t>Selesai</t>
         </is>
       </c>
-      <c r="J5" s="10" t="inlineStr">
+      <c r="J5" s="12" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
@@ -1227,17 +1259,17 @@
           <t>0.2</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Fase 0 - Verifikasi Meja</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>Protokol v2 + byte rem</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>protocol.h / protocol.py / protocol.md kembar, paket 12 byte</t>
         </is>
@@ -1265,7 +1297,7 @@
           <t>Selesai</t>
         </is>
       </c>
-      <c r="J6" s="10" t="inlineStr">
+      <c r="J6" s="12" t="inlineStr">
         <is>
           <t>docs/protocol.md</t>
         </is>
@@ -1277,17 +1309,17 @@
           <t>0.3</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Fase 0 - Verifikasi Meja</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Kalibrasi stir PXN V9 (V9GEN2)</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>calibration.yaml: h_pattern, gigi 1-6 di btn 16-21, R di btn 22</t>
         </is>
@@ -1315,7 +1347,7 @@
           <t>Selesai</t>
         </is>
       </c>
-      <c r="J7" s="10" t="inlineStr">
+      <c r="J7" s="12" t="inlineStr">
         <is>
           <t>ground/calibration.yaml</t>
         </is>
@@ -1327,17 +1359,17 @@
           <t>0.4</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Fase 0 - Verifikasi Meja</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>Port kamera ke XIAO ESP32S3 Sense</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>16/16 pin cocok definisi resmi core; kompilasi 28% flash</t>
         </is>
@@ -1365,7 +1397,7 @@
           <t>Selesai</t>
         </is>
       </c>
-      <c r="J8" s="10" t="inlineStr">
+      <c r="J8" s="12" t="inlineStr">
         <is>
           <t>firmware/rc_cam_esp32</t>
         </is>
@@ -1377,17 +1409,17 @@
           <t>0.5</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Fase 0 - Verifikasi Meja</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Isi kredensial WiFi kedua firmware</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>SSID RCCar terisi di config.h dan rc_cam_esp32.ino</t>
         </is>
@@ -1415,7 +1447,7 @@
           <t>Selesai</t>
         </is>
       </c>
-      <c r="J9" s="10" t="inlineStr">
+      <c r="J9" s="12" t="inlineStr">
         <is>
           <t>firmware/</t>
         </is>
@@ -1427,17 +1459,17 @@
           <t>1.1</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Fase 1 - Wiring &amp; Daya</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>Setel step-down #1 ke 12,0 V TANPA beban</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Multimeter baca 12,0 +/- 0,1 V sebelum disambung ke apa pun</t>
         </is>
@@ -1465,7 +1497,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J10" s="10" t="inlineStr">
+      <c r="J10" s="12" t="inlineStr">
         <is>
           <t>wiring 2</t>
         </is>
@@ -1477,17 +1509,17 @@
           <t>1.2</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Fase 1 - Wiring &amp; Daya</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>Setel step-down #2 ke 5,0 V TANPA beban</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Multimeter baca 5,0 +/- 0,05 V sebelum disambung ke apa pun</t>
         </is>
@@ -1515,7 +1547,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J11" s="10" t="inlineStr">
+      <c r="J11" s="12" t="inlineStr">
         <is>
           <t>wiring 2</t>
         </is>
@@ -1527,17 +1559,17 @@
           <t>1.3</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Fase 1 - Wiring &amp; Daya</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>Lepas jumper ENA di L298N</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Jumper fisik terlepas. Kalau tidak, PWM tidak berefek sama sekali</t>
         </is>
@@ -1565,7 +1597,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J12" s="10" t="inlineStr">
+      <c r="J12" s="12" t="inlineStr">
         <is>
           <t>wiring 4</t>
         </is>
@@ -1577,17 +1609,17 @@
           <t>1.4</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Fase 1 - Wiring &amp; Daya</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>Lepas jumper 5V di L298N</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>Regulator on-board mati; 5V hanya dari step-down #2</t>
         </is>
@@ -1615,7 +1647,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J13" s="10" t="inlineStr">
+      <c r="J13" s="12" t="inlineStr">
         <is>
           <t>wiring 4</t>
         </is>
@@ -1627,17 +1659,17 @@
           <t>1.5</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>Fase 1 - Wiring &amp; Daya</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>Pindah sinyal servo GPIO 34 -&gt; GPIO 13</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>GPIO 34 input-only, tidak bisa mengeluarkan pulsa servo</t>
         </is>
@@ -1665,7 +1697,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J14" s="10" t="inlineStr">
+      <c r="J14" s="12" t="inlineStr">
         <is>
           <t>wiring 3</t>
         </is>
@@ -1677,17 +1709,17 @@
           <t>1.6</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Fase 1 - Wiring &amp; Daya</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>Pasang pulldown 10k di ENA, IN1, IN2</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>3 resistor ke GND; menjamin motor mati saat ESP32 boot</t>
         </is>
@@ -1715,7 +1747,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J15" s="10" t="inlineStr">
+      <c r="J15" s="12" t="inlineStr">
         <is>
           <t>wiring 4</t>
         </is>
@@ -1727,17 +1759,17 @@
           <t>1.7</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Fase 1 - Wiring &amp; Daya</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
         <is>
           <t>Rakit pembagi tegangan 100k/22k ke GPIO 34</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>Ukur ~3,03 V saat 4S penuh (16,8 V). Tambah 100nF ke GND</t>
         </is>
@@ -1765,7 +1797,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J16" s="10" t="inlineStr">
+      <c r="J16" s="12" t="inlineStr">
         <is>
           <t>wiring 6</t>
         </is>
@@ -1777,17 +1809,17 @@
           <t>1.8</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>Fase 1 - Wiring &amp; Daya</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="C17" s="12" t="inlineStr">
         <is>
           <t>Star ground: semua GND ke SATU titik</t>
         </is>
       </c>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>Kedua step-down, L298N, servo, kedua ESP32, pembagi</t>
         </is>
@@ -1815,7 +1847,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J17" s="10" t="inlineStr">
+      <c r="J17" s="12" t="inlineStr">
         <is>
           <t>wiring 2</t>
         </is>
@@ -1827,17 +1859,17 @@
           <t>1.9</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>Fase 1 - Wiring &amp; Daya</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr">
         <is>
           <t>Elko 470uF di terminal Vs L298N</t>
         </is>
       </c>
-      <c r="D18" s="10" t="inlineStr">
+      <c r="D18" s="12" t="inlineStr">
         <is>
           <t>Terpasang, polaritas benar</t>
         </is>
@@ -1865,7 +1897,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J18" s="10" t="inlineStr">
+      <c r="J18" s="12" t="inlineStr">
         <is>
           <t>wiring 2</t>
         </is>
@@ -1877,17 +1909,17 @@
           <t>1.10</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>Fase 1 - Wiring &amp; Daya</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>Elko 1000uF di jalur 5V servo</t>
         </is>
       </c>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="D19" s="12" t="inlineStr">
         <is>
           <t>SEDEKAT MUNGKIN ke konektor servo, bukan di step-down</t>
         </is>
@@ -1915,7 +1947,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J19" s="10" t="inlineStr">
+      <c r="J19" s="12" t="inlineStr">
         <is>
           <t>wiring 2</t>
         </is>
@@ -1927,17 +1959,17 @@
           <t>1.11</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>Fase 1 - Wiring &amp; Daya</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C20" s="12" t="inlineStr">
         <is>
           <t>Elko 470uF + 100nF di 5V kamera</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="D20" s="12" t="inlineStr">
         <is>
           <t>Sedekat mungkin ke XIAO. Cegah brownout saat WiFi transmit</t>
         </is>
@@ -1965,7 +1997,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J20" s="10" t="inlineStr">
+      <c r="J20" s="12" t="inlineStr">
         <is>
           <t>wiring 7a</t>
         </is>
@@ -1977,17 +2009,17 @@
           <t>1.12</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>Fase 1 - Wiring &amp; Daya</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>Tiga keramik 100nF di badan motor</t>
         </is>
       </c>
-      <c r="D21" s="10" t="inlineStr">
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>2 terminal + masing-masing ke casing. Redam noise ke WiFi/video</t>
         </is>
@@ -2015,7 +2047,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J21" s="10" t="inlineStr">
+      <c r="J21" s="12" t="inlineStr">
         <is>
           <t>wiring 4</t>
         </is>
@@ -2027,17 +2059,17 @@
           <t>1.13</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>Fase 1 - Wiring &amp; Daya</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr">
+      <c r="C22" s="12" t="inlineStr">
         <is>
           <t>Pasang antena eksternal u.FL di XIAO</t>
         </is>
       </c>
-      <c r="D22" s="10" t="inlineStr">
+      <c r="D22" s="12" t="inlineStr">
         <is>
           <t>Tanpa ini jangkauan jauh lebih pendek</t>
         </is>
@@ -2065,7 +2097,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J22" s="10" t="inlineStr">
+      <c r="J22" s="12" t="inlineStr">
         <is>
           <t>wiring 7a</t>
         </is>
@@ -2127,17 +2159,17 @@
           <t>2.1</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>Fase 2 - Flash &amp; Bench</t>
         </is>
       </c>
-      <c r="C24" s="10" t="inlineStr">
+      <c r="C24" s="12" t="inlineStr">
         <is>
           <t>Nyalakan hotspot RCCar di laptop</t>
         </is>
       </c>
-      <c r="D24" s="10" t="inlineStr">
+      <c r="D24" s="12" t="inlineStr">
         <is>
           <t>SSID RCCar aktif, subnet 192.168.137.x, gateway .1</t>
         </is>
@@ -2147,7 +2179,7 @@
       </c>
       <c r="F24" s="16" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="G24" s="16" t="inlineStr">
@@ -2165,7 +2197,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J24" s="10" t="inlineStr">
+      <c r="J24" s="12" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
@@ -2177,17 +2209,17 @@
           <t>2.2</t>
         </is>
       </c>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>Fase 2 - Flash &amp; Bench</t>
         </is>
       </c>
-      <c r="C25" s="10" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>Flash rc_car_esp32 (board: ESP32 Dev Module)</t>
         </is>
       </c>
-      <c r="D25" s="10" t="inlineStr">
+      <c r="D25" s="12" t="inlineStr">
         <is>
           <t>Upload sukses tanpa error</t>
         </is>
@@ -2197,7 +2229,7 @@
       </c>
       <c r="F25" s="16" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="G25" s="16" t="inlineStr">
@@ -2215,7 +2247,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J25" s="10" t="inlineStr">
+      <c r="J25" s="12" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
@@ -2247,7 +2279,7 @@
       </c>
       <c r="F26" s="17" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="G26" s="17" t="inlineStr">
@@ -2277,17 +2309,17 @@
           <t>2.4</t>
         </is>
       </c>
-      <c r="B27" s="10" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>Fase 2 - Flash &amp; Bench</t>
         </is>
       </c>
-      <c r="C27" s="10" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
         <is>
           <t>Flash rc_cam_esp32 (XIAO, PSRAM = OPI PSRAM)</t>
         </is>
       </c>
-      <c r="D27" s="10" t="inlineStr">
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>PSRAM WAJIB diubah dari Disabled ke OPI PSRAM</t>
         </is>
@@ -2297,7 +2329,7 @@
       </c>
       <c r="F27" s="16" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="G27" s="16" t="inlineStr">
@@ -2315,7 +2347,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J27" s="10" t="inlineStr">
+      <c r="J27" s="12" t="inlineStr">
         <is>
           <t>camera_pins.h</t>
         </is>
@@ -2347,7 +2379,7 @@
       </c>
       <c r="F28" s="17" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="G28" s="17" t="inlineStr">
@@ -2377,17 +2409,17 @@
           <t>2.6</t>
         </is>
       </c>
-      <c r="B29" s="10" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>Fase 2 - Flash &amp; Bench</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr">
+      <c r="C29" s="12" t="inlineStr">
         <is>
           <t>Uji stream kamera di browser dulu</t>
         </is>
       </c>
-      <c r="D29" s="10" t="inlineStr">
+      <c r="D29" s="12" t="inlineStr">
         <is>
           <t>http://192.168.137.60/ gambar muncul dan stabil, sebelum ground station</t>
         </is>
@@ -2397,7 +2429,7 @@
       </c>
       <c r="F29" s="16" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="G29" s="16" t="inlineStr">
@@ -2415,7 +2447,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J29" s="10" t="inlineStr">
+      <c r="J29" s="12" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
@@ -2427,17 +2459,17 @@
           <t>2.7</t>
         </is>
       </c>
-      <c r="B30" s="10" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>Fase 2 - Flash &amp; Bench</t>
         </is>
       </c>
-      <c r="C30" s="10" t="inlineStr">
+      <c r="C30" s="12" t="inlineStr">
         <is>
           <t>Kalibrasi VBAT_DIVIDER_RATIO</t>
         </is>
       </c>
-      <c r="D30" s="10" t="inlineStr">
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>Tegangan di HUD cocok multimeter +/- 0,1 V</t>
         </is>
@@ -2465,7 +2497,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J30" s="10" t="inlineStr">
+      <c r="J30" s="12" t="inlineStr">
         <is>
           <t>wiring 6</t>
         </is>
@@ -2477,17 +2509,17 @@
           <t>2.8</t>
         </is>
       </c>
-      <c r="B31" s="10" t="inlineStr">
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>Fase 2 - Flash &amp; Bench</t>
         </is>
       </c>
-      <c r="C31" s="10" t="inlineStr">
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>Uji servo saja, motor BELUM disambung</t>
         </is>
       </c>
-      <c r="D31" s="10" t="inlineStr">
+      <c r="D31" s="12" t="inlineStr">
         <is>
           <t>Servo bergerak halus mengikuti stir</t>
         </is>
@@ -2515,7 +2547,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J31" s="10" t="inlineStr">
+      <c r="J31" s="12" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
@@ -2527,17 +2559,17 @@
           <t>2.9</t>
         </is>
       </c>
-      <c r="B32" s="10" t="inlineStr">
+      <c r="B32" s="12" t="inlineStr">
         <is>
           <t>Fase 2 - Flash &amp; Bench</t>
         </is>
       </c>
-      <c r="C32" s="10" t="inlineStr">
+      <c r="C32" s="12" t="inlineStr">
         <is>
           <t>Setel SERVO_MIN_US / SERVO_MAX_US bertahap</t>
         </is>
       </c>
-      <c r="D32" s="10" t="inlineStr">
+      <c r="D32" s="12" t="inlineStr">
         <is>
           <t>Mulai 1300/1700, lebarkan 50us tiap kali. Berhenti saat mulai mendengung</t>
         </is>
@@ -2565,7 +2597,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J32" s="10" t="inlineStr">
+      <c r="J32" s="12" t="inlineStr">
         <is>
           <t>wiring 5</t>
         </is>
@@ -2577,17 +2609,17 @@
           <t>2.10</t>
         </is>
       </c>
-      <c r="B33" s="10" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>Fase 2 - Flash &amp; Bench</t>
         </is>
       </c>
-      <c r="C33" s="10" t="inlineStr">
+      <c r="C33" s="12" t="inlineStr">
         <is>
           <t>Sambung motor, RODA DI UDARA, max_forward 0.30</t>
         </is>
       </c>
-      <c r="D33" s="10" t="inlineStr">
+      <c r="D33" s="12" t="inlineStr">
         <is>
           <t>Motor berputar maju terkendali</t>
         </is>
@@ -2615,7 +2647,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J33" s="10" t="inlineStr">
+      <c r="J33" s="12" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
@@ -2627,17 +2659,17 @@
           <t>2.11</t>
         </is>
       </c>
-      <c r="B34" s="10" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>Fase 2 - Flash &amp; Bench</t>
         </is>
       </c>
-      <c r="C34" s="10" t="inlineStr">
+      <c r="C34" s="12" t="inlineStr">
         <is>
           <t>Verifikasi arah maju/mundur</t>
         </is>
       </c>
-      <c r="D34" s="10" t="inlineStr">
+      <c r="D34" s="12" t="inlineStr">
         <is>
           <t>Kalau terbalik: tukar OUT1 dan OUT2, jangan diubah lewat program</t>
         </is>
@@ -2665,7 +2697,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J34" s="10" t="inlineStr">
+      <c r="J34" s="12" t="inlineStr">
         <is>
           <t>wiring 4</t>
         </is>
@@ -2677,17 +2709,17 @@
           <t>2.12</t>
         </is>
       </c>
-      <c r="B35" s="10" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>Fase 2 - Flash &amp; Bench</t>
         </is>
       </c>
-      <c r="C35" s="10" t="inlineStr">
+      <c r="C35" s="12" t="inlineStr">
         <is>
           <t>Uji tuas gigi N / 1-6 / R</t>
         </is>
       </c>
-      <c r="D35" s="10" t="inlineStr">
+      <c r="D35" s="12" t="inlineStr">
         <is>
           <t>N tidak jalan; harus di N untuk arm; R mundur; tiap gigi batasi kecepatan</t>
         </is>
@@ -2715,7 +2747,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J35" s="10" t="inlineStr">
+      <c r="J35" s="12" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
@@ -2727,17 +2759,17 @@
           <t>2.13</t>
         </is>
       </c>
-      <c r="B36" s="10" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>Fase 2 - Flash &amp; Bench</t>
         </is>
       </c>
-      <c r="C36" s="10" t="inlineStr">
+      <c r="C36" s="12" t="inlineStr">
         <is>
           <t>Uji pedal rem (sekarang benar-benar mengerem)</t>
         </is>
       </c>
-      <c r="D36" s="10" t="inlineStr">
+      <c r="D36" s="12" t="inlineStr">
         <is>
           <t>Motor mengerem, bukan berbalik arah seperti versi lama</t>
         </is>
@@ -2765,7 +2797,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J36" s="10" t="inlineStr">
+      <c r="J36" s="12" t="inlineStr">
         <is>
           <t>protocol 3</t>
         </is>
@@ -2777,17 +2809,17 @@
           <t>2.14</t>
         </is>
       </c>
-      <c r="B37" s="10" t="inlineStr">
+      <c r="B37" s="12" t="inlineStr">
         <is>
           <t>Fase 2 - Flash &amp; Bench</t>
         </is>
       </c>
-      <c r="C37" s="10" t="inlineStr">
+      <c r="C37" s="12" t="inlineStr">
         <is>
           <t>Cek suhu L298N &amp; step-down setelah 30 detik</t>
         </is>
       </c>
-      <c r="D37" s="10" t="inlineStr">
+      <c r="D37" s="12" t="inlineStr">
         <is>
           <t>Hangat wajar. Panas = ada masalah, hentikan dan periksa</t>
         </is>
@@ -2815,7 +2847,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J37" s="10" t="inlineStr">
+      <c r="J37" s="12" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
@@ -2847,7 +2879,7 @@
       </c>
       <c r="F38" s="17" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="G38" s="17" t="inlineStr">
@@ -2897,7 +2929,7 @@
       </c>
       <c r="F39" s="17" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="G39" s="17" t="inlineStr">
@@ -2947,7 +2979,7 @@
       </c>
       <c r="F40" s="17" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="G40" s="17" t="inlineStr">
@@ -2977,17 +3009,17 @@
           <t>3.4</t>
         </is>
       </c>
-      <c r="B41" s="10" t="inlineStr">
+      <c r="B41" s="12" t="inlineStr">
         <is>
           <t>Fase 3 - Failsafe &amp; Integrasi</t>
         </is>
       </c>
-      <c r="C41" s="10" t="inlineStr">
+      <c r="C41" s="12" t="inlineStr">
         <is>
           <t>Ukur PING di HUD</t>
         </is>
       </c>
-      <c r="D41" s="10" t="inlineStr">
+      <c r="D41" s="12" t="inlineStr">
         <is>
           <t>Target &lt; 30 ms di jaringan hotspot yang sehat</t>
         </is>
@@ -2997,7 +3029,7 @@
       </c>
       <c r="F41" s="16" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="G41" s="16" t="inlineStr">
@@ -3015,7 +3047,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J41" s="10" t="inlineStr">
+      <c r="J41" s="12" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
@@ -3027,17 +3059,17 @@
           <t>3.5</t>
         </is>
       </c>
-      <c r="B42" s="10" t="inlineStr">
+      <c r="B42" s="12" t="inlineStr">
         <is>
           <t>Fase 3 - Failsafe &amp; Integrasi</t>
         </is>
       </c>
-      <c r="C42" s="10" t="inlineStr">
+      <c r="C42" s="12" t="inlineStr">
         <is>
           <t>Ukur VIDEO fps di HUD</t>
         </is>
       </c>
-      <c r="D42" s="10" t="inlineStr">
+      <c r="D42" s="12" t="inlineStr">
         <is>
           <t>Target &gt;= 15 fps pada VGA 640x480</t>
         </is>
@@ -3047,7 +3079,7 @@
       </c>
       <c r="F42" s="16" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="G42" s="16" t="inlineStr">
@@ -3065,7 +3097,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J42" s="10" t="inlineStr">
+      <c r="J42" s="12" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
@@ -3077,17 +3109,17 @@
           <t>3.6</t>
         </is>
       </c>
-      <c r="B43" s="10" t="inlineStr">
+      <c r="B43" s="12" t="inlineStr">
         <is>
           <t>Fase 3 - Failsafe &amp; Integrasi</t>
         </is>
       </c>
-      <c r="C43" s="10" t="inlineStr">
+      <c r="C43" s="12" t="inlineStr">
         <is>
           <t>Uji jangkauan bertahap 10 / 20 / 30 m</t>
         </is>
       </c>
-      <c r="D43" s="10" t="inlineStr">
+      <c r="D43" s="12" t="inlineStr">
         <is>
           <t>Catat PING, fps, dan RSSI tiap jarak. Cari batas amannya</t>
         </is>
@@ -3097,7 +3129,7 @@
       </c>
       <c r="F43" s="16" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="G43" s="16" t="inlineStr">
@@ -3115,7 +3147,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J43" s="10" t="inlineStr">
+      <c r="J43" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3127,17 +3159,17 @@
           <t>3.7</t>
         </is>
       </c>
-      <c r="B44" s="10" t="inlineStr">
+      <c r="B44" s="12" t="inlineStr">
         <is>
           <t>Fase 3 - Failsafe &amp; Integrasi</t>
         </is>
       </c>
-      <c r="C44" s="10" t="inlineStr">
+      <c r="C44" s="12" t="inlineStr">
         <is>
           <t>Uji tombol stop darurat</t>
         </is>
       </c>
-      <c r="D44" s="10" t="inlineStr">
+      <c r="D44" s="12" t="inlineStr">
         <is>
           <t>Tombol E dan tombol estop di stir menghentikan motor seketika</t>
         </is>
@@ -3147,7 +3179,7 @@
       </c>
       <c r="F44" s="16" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="G44" s="16" t="inlineStr">
@@ -3165,7 +3197,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J44" s="10" t="inlineStr">
+      <c r="J44" s="12" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
@@ -3177,17 +3209,17 @@
           <t>4.1</t>
         </is>
       </c>
-      <c r="B45" s="10" t="inlineStr">
+      <c r="B45" s="12" t="inlineStr">
         <is>
           <t>Fase 4 - Uji Lantai &amp; Tuning</t>
         </is>
       </c>
-      <c r="C45" s="10" t="inlineStr">
+      <c r="C45" s="12" t="inlineStr">
         <is>
           <t>Turunkan ke lantai, ruang terbuka, max_forward 0.30</t>
         </is>
       </c>
-      <c r="D45" s="10" t="inlineStr">
+      <c r="D45" s="12" t="inlineStr">
         <is>
           <t>Mobil jalan terkendali, tidak ada perilaku kejut</t>
         </is>
@@ -3197,7 +3229,7 @@
       </c>
       <c r="F45" s="16" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="G45" s="16" t="inlineStr">
@@ -3215,7 +3247,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J45" s="10" t="inlineStr">
+      <c r="J45" s="12" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
@@ -3227,17 +3259,17 @@
           <t>4.2</t>
         </is>
       </c>
-      <c r="B46" s="10" t="inlineStr">
+      <c r="B46" s="12" t="inlineStr">
         <is>
           <t>Fase 4 - Uji Lantai &amp; Tuning</t>
         </is>
       </c>
-      <c r="C46" s="10" t="inlineStr">
+      <c r="C46" s="12" t="inlineStr">
         <is>
           <t>Setel trim stir sampai lurus, simpan dengan F5</t>
         </is>
       </c>
-      <c r="D46" s="10" t="inlineStr">
+      <c r="D46" s="12" t="inlineStr">
         <is>
           <t>Mobil berjalan lurus tanpa dikoreksi terus</t>
         </is>
@@ -3247,7 +3279,7 @@
       </c>
       <c r="F46" s="16" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="G46" s="16" t="inlineStr">
@@ -3265,7 +3297,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J46" s="10" t="inlineStr">
+      <c r="J46" s="12" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
@@ -3277,17 +3309,17 @@
           <t>4.3</t>
         </is>
       </c>
-      <c r="B47" s="10" t="inlineStr">
+      <c r="B47" s="12" t="inlineStr">
         <is>
           <t>Fase 4 - Uji Lantai &amp; Tuning</t>
         </is>
       </c>
-      <c r="C47" s="10" t="inlineStr">
+      <c r="C47" s="12" t="inlineStr">
         <is>
           <t>Naikkan max_forward bertahap 0.30 -&gt; 0.50 -&gt; 0.70</t>
         </is>
       </c>
-      <c r="D47" s="10" t="inlineStr">
+      <c r="D47" s="12" t="inlineStr">
         <is>
           <t>Tetap terkendali di tiap tahap sebelum naik lagi</t>
         </is>
@@ -3297,7 +3329,7 @@
       </c>
       <c r="F47" s="16" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="G47" s="16" t="inlineStr">
@@ -3315,7 +3347,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J47" s="10" t="inlineStr">
+      <c r="J47" s="12" t="inlineStr">
         <is>
           <t>config.yaml</t>
         </is>
@@ -3327,17 +3359,17 @@
           <t>4.4</t>
         </is>
       </c>
-      <c r="B48" s="10" t="inlineStr">
+      <c r="B48" s="12" t="inlineStr">
         <is>
           <t>Fase 4 - Uji Lantai &amp; Tuning</t>
         </is>
       </c>
-      <c r="C48" s="10" t="inlineStr">
+      <c r="C48" s="12" t="inlineStr">
         <is>
           <t>Setel gear_ratios sesuai rasa berkendara</t>
         </is>
       </c>
-      <c r="D48" s="10" t="inlineStr">
+      <c r="D48" s="12" t="inlineStr">
         <is>
           <t>Gigi 1 berguna untuk manuver rapat, gigi atas untuk lurus</t>
         </is>
@@ -3347,7 +3379,7 @@
       </c>
       <c r="F48" s="16" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="G48" s="16" t="inlineStr">
@@ -3365,7 +3397,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J48" s="10" t="inlineStr">
+      <c r="J48" s="12" t="inlineStr">
         <is>
           <t>config.yaml</t>
         </is>
@@ -3377,17 +3409,17 @@
           <t>4.5</t>
         </is>
       </c>
-      <c r="B49" s="10" t="inlineStr">
+      <c r="B49" s="12" t="inlineStr">
         <is>
           <t>Fase 4 - Uji Lantai &amp; Tuning</t>
         </is>
       </c>
-      <c r="C49" s="10" t="inlineStr">
+      <c r="C49" s="12" t="inlineStr">
         <is>
           <t>Setel expo stir dan gas</t>
         </is>
       </c>
-      <c r="D49" s="10" t="inlineStr">
+      <c r="D49" s="12" t="inlineStr">
         <is>
           <t>Respons halus di tengah, tetap penuh di ujung</t>
         </is>
@@ -3397,7 +3429,7 @@
       </c>
       <c r="F49" s="16" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="G49" s="16" t="inlineStr">
@@ -3415,7 +3447,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J49" s="10" t="inlineStr">
+      <c r="J49" s="12" t="inlineStr">
         <is>
           <t>config.yaml</t>
         </is>
@@ -3427,17 +3459,17 @@
           <t>4.6</t>
         </is>
       </c>
-      <c r="B50" s="10" t="inlineStr">
+      <c r="B50" s="12" t="inlineStr">
         <is>
           <t>Fase 4 - Uji Lantai &amp; Tuning</t>
         </is>
       </c>
-      <c r="C50" s="10" t="inlineStr">
+      <c r="C50" s="12" t="inlineStr">
         <is>
           <t>Ukur waktu jalan sampai 14,0 V</t>
         </is>
       </c>
-      <c r="D50" s="10" t="inlineStr">
+      <c r="D50" s="12" t="inlineStr">
         <is>
           <t>Catat menit sebenarnya. Perkiraan 5-8 menit dengan 4S 850 mAh</t>
         </is>
@@ -3447,7 +3479,7 @@
       </c>
       <c r="F50" s="16" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="G50" s="16" t="inlineStr">
@@ -3465,7 +3497,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J50" s="10" t="inlineStr">
+      <c r="J50" s="12" t="inlineStr">
         <is>
           <t>wiring 2</t>
         </is>
@@ -3477,17 +3509,17 @@
           <t>5.1</t>
         </is>
       </c>
-      <c r="B51" s="10" t="inlineStr">
+      <c r="B51" s="12" t="inlineStr">
         <is>
           <t>Fase 5 - Pindah ke LattePanda</t>
         </is>
       </c>
-      <c r="C51" s="10" t="inlineStr">
+      <c r="C51" s="12" t="inlineStr">
         <is>
           <t>Install Python 3 di LattePanda</t>
         </is>
       </c>
-      <c r="D51" s="10" t="inlineStr">
+      <c r="D51" s="12" t="inlineStr">
         <is>
           <t>python --version berjalan</t>
         </is>
@@ -3497,7 +3529,7 @@
       </c>
       <c r="F51" s="16" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="G51" s="16" t="inlineStr">
@@ -3515,7 +3547,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J51" s="10" t="inlineStr">
+      <c r="J51" s="12" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
@@ -3527,17 +3559,17 @@
           <t>5.2</t>
         </is>
       </c>
-      <c r="B52" s="10" t="inlineStr">
+      <c r="B52" s="12" t="inlineStr">
         <is>
           <t>Fase 5 - Pindah ke LattePanda</t>
         </is>
       </c>
-      <c r="C52" s="10" t="inlineStr">
+      <c r="C52" s="12" t="inlineStr">
         <is>
           <t>Salin folder proyek ke LattePanda</t>
         </is>
       </c>
-      <c r="D52" s="10" t="inlineStr">
+      <c r="D52" s="12" t="inlineStr">
         <is>
           <t>Seluruh folder RC Car tersalin</t>
         </is>
@@ -3547,7 +3579,7 @@
       </c>
       <c r="F52" s="16" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="G52" s="16" t="inlineStr">
@@ -3565,7 +3597,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J52" s="10" t="inlineStr">
+      <c r="J52" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3577,17 +3609,17 @@
           <t>5.3</t>
         </is>
       </c>
-      <c r="B53" s="10" t="inlineStr">
+      <c r="B53" s="12" t="inlineStr">
         <is>
           <t>Fase 5 - Pindah ke LattePanda</t>
         </is>
       </c>
-      <c r="C53" s="10" t="inlineStr">
+      <c r="C53" s="12" t="inlineStr">
         <is>
           <t>pip install -r ground/requirements.txt</t>
         </is>
       </c>
-      <c r="D53" s="10" t="inlineStr">
+      <c r="D53" s="12" t="inlineStr">
         <is>
           <t>pygame dan PyYAML terpasang</t>
         </is>
@@ -3597,7 +3629,7 @@
       </c>
       <c r="F53" s="16" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="G53" s="16" t="inlineStr">
@@ -3615,7 +3647,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J53" s="10" t="inlineStr">
+      <c r="J53" s="12" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
@@ -3627,17 +3659,17 @@
           <t>5.4</t>
         </is>
       </c>
-      <c r="B54" s="10" t="inlineStr">
+      <c r="B54" s="12" t="inlineStr">
         <is>
           <t>Fase 5 - Pindah ke LattePanda</t>
         </is>
       </c>
-      <c r="C54" s="10" t="inlineStr">
+      <c r="C54" s="12" t="inlineStr">
         <is>
           <t>Jalankan calibrate.py di LattePanda</t>
         </is>
       </c>
-      <c r="D54" s="10" t="inlineStr">
+      <c r="D54" s="12" t="inlineStr">
         <is>
           <t>calibration.yaml baru; enumerasi USB bisa berbeda dari laptop</t>
         </is>
@@ -3647,7 +3679,7 @@
       </c>
       <c r="F54" s="16" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="G54" s="16" t="inlineStr">
@@ -3665,7 +3697,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J54" s="10" t="inlineStr">
+      <c r="J54" s="12" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
@@ -3677,17 +3709,17 @@
           <t>5.5</t>
         </is>
       </c>
-      <c r="B55" s="10" t="inlineStr">
+      <c r="B55" s="12" t="inlineStr">
         <is>
           <t>Fase 5 - Pindah ke LattePanda</t>
         </is>
       </c>
-      <c r="C55" s="10" t="inlineStr">
+      <c r="C55" s="12" t="inlineStr">
         <is>
           <t>Pindahkan hotspot RCCar ke LattePanda</t>
         </is>
       </c>
-      <c r="D55" s="10" t="inlineStr">
+      <c r="D55" s="12" t="inlineStr">
         <is>
           <t>SSID dan subnet sama supaya IP statis tetap cocok</t>
         </is>
@@ -3697,7 +3729,7 @@
       </c>
       <c r="F55" s="16" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="G55" s="16" t="inlineStr">
@@ -3715,7 +3747,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J55" s="10" t="inlineStr">
+      <c r="J55" s="12" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
@@ -3747,7 +3779,7 @@
       </c>
       <c r="F56" s="17" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="G56" s="17" t="inlineStr">
@@ -3777,17 +3809,17 @@
           <t>6.1</t>
         </is>
       </c>
-      <c r="B57" s="10" t="inlineStr">
+      <c r="B57" s="12" t="inlineStr">
         <is>
           <t>Fase 6 - Finalisasi</t>
         </is>
       </c>
-      <c r="C57" s="10" t="inlineStr">
+      <c r="C57" s="12" t="inlineStr">
         <is>
           <t>Rapikan dan ikat seluruh kabel</t>
         </is>
       </c>
-      <c r="D57" s="10" t="inlineStr">
+      <c r="D57" s="12" t="inlineStr">
         <is>
           <t>Tidak ada kabel menjuntai ke roda atau gardan</t>
         </is>
@@ -3797,7 +3829,7 @@
       </c>
       <c r="F57" s="16" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G57" s="16" t="inlineStr">
@@ -3815,7 +3847,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J57" s="10" t="inlineStr">
+      <c r="J57" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3827,17 +3859,17 @@
           <t>6.2</t>
         </is>
       </c>
-      <c r="B58" s="10" t="inlineStr">
+      <c r="B58" s="12" t="inlineStr">
         <is>
           <t>Fase 6 - Finalisasi</t>
         </is>
       </c>
-      <c r="C58" s="10" t="inlineStr">
+      <c r="C58" s="12" t="inlineStr">
         <is>
           <t>Pasang semua modul permanen di sasis</t>
         </is>
       </c>
-      <c r="D58" s="10" t="inlineStr">
+      <c r="D58" s="12" t="inlineStr">
         <is>
           <t>Tidak bergeser saat menikung atau menabrak</t>
         </is>
@@ -3847,7 +3879,7 @@
       </c>
       <c r="F58" s="16" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G58" s="16" t="inlineStr">
@@ -3865,7 +3897,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J58" s="10" t="inlineStr">
+      <c r="J58" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3877,17 +3909,17 @@
           <t>6.3</t>
         </is>
       </c>
-      <c r="B59" s="10" t="inlineStr">
+      <c r="B59" s="12" t="inlineStr">
         <is>
           <t>Fase 6 - Finalisasi</t>
         </is>
       </c>
-      <c r="C59" s="10" t="inlineStr">
+      <c r="C59" s="12" t="inlineStr">
         <is>
           <t>Foto wiring aktual dari beberapa sudut</t>
         </is>
       </c>
-      <c r="D59" s="10" t="inlineStr">
+      <c r="D59" s="12" t="inlineStr">
         <is>
           <t>Arsip visual untuk duplikasi nanti</t>
         </is>
@@ -3897,7 +3929,7 @@
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G59" s="16" t="inlineStr">
@@ -3915,7 +3947,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J59" s="10" t="inlineStr">
+      <c r="J59" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3927,17 +3959,17 @@
           <t>6.4</t>
         </is>
       </c>
-      <c r="B60" s="10" t="inlineStr">
+      <c r="B60" s="12" t="inlineStr">
         <is>
           <t>Fase 6 - Finalisasi</t>
         </is>
       </c>
-      <c r="C60" s="10" t="inlineStr">
+      <c r="C60" s="12" t="inlineStr">
         <is>
           <t>Perbarui docs/wiring.md sesuai hardware nyata</t>
         </is>
       </c>
-      <c r="D60" s="10" t="inlineStr">
+      <c r="D60" s="12" t="inlineStr">
         <is>
           <t>Dokumen cocok 100% dengan yang terpasang</t>
         </is>
@@ -3947,7 +3979,7 @@
       </c>
       <c r="F60" s="16" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G60" s="16" t="inlineStr">
@@ -3965,7 +3997,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J60" s="10" t="inlineStr">
+      <c r="J60" s="12" t="inlineStr">
         <is>
           <t>docs/wiring.md</t>
         </is>
@@ -3977,17 +4009,17 @@
           <t>6.5</t>
         </is>
       </c>
-      <c r="B61" s="10" t="inlineStr">
+      <c r="B61" s="12" t="inlineStr">
         <is>
           <t>Fase 6 - Finalisasi</t>
         </is>
       </c>
-      <c r="C61" s="10" t="inlineStr">
+      <c r="C61" s="12" t="inlineStr">
         <is>
           <t>Catat nilai tuning final di config.yaml</t>
         </is>
       </c>
-      <c r="D61" s="10" t="inlineStr">
+      <c r="D61" s="12" t="inlineStr">
         <is>
           <t>Nilai yang benar-benar terbukti di lapangan</t>
         </is>
@@ -3997,7 +4029,7 @@
       </c>
       <c r="F61" s="16" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G61" s="16" t="inlineStr">
@@ -4015,7 +4047,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J61" s="10" t="inlineStr">
+      <c r="J61" s="12" t="inlineStr">
         <is>
           <t>config.yaml</t>
         </is>
@@ -4027,17 +4059,17 @@
           <t>6.6</t>
         </is>
       </c>
-      <c r="B62" s="10" t="inlineStr">
+      <c r="B62" s="12" t="inlineStr">
         <is>
           <t>Fase 6 - Finalisasi</t>
         </is>
       </c>
-      <c r="C62" s="10" t="inlineStr">
+      <c r="C62" s="12" t="inlineStr">
         <is>
           <t>Backup proyek (git init + commit atau arsip)</t>
         </is>
       </c>
-      <c r="D62" s="10" t="inlineStr">
+      <c r="D62" s="12" t="inlineStr">
         <is>
           <t>Ada salinan yang bisa dikembalikan kalau rusak</t>
         </is>
@@ -4047,7 +4079,7 @@
       </c>
       <c r="F62" s="16" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G62" s="16" t="inlineStr">
@@ -4065,7 +4097,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J62" s="10" t="inlineStr">
+      <c r="J62" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4097,7 +4129,7 @@
       </c>
       <c r="F63" s="17" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G63" s="17" t="inlineStr">
@@ -4127,17 +4159,17 @@
           <t>7.1</t>
         </is>
       </c>
-      <c r="B64" s="10" t="inlineStr">
+      <c r="B64" s="12" t="inlineStr">
         <is>
           <t>Fase 7 - Duplikasi &amp; Produksi</t>
         </is>
       </c>
-      <c r="C64" s="10" t="inlineStr">
+      <c r="C64" s="12" t="inlineStr">
         <is>
           <t>Susun BOM final: harga + sumber beli</t>
         </is>
       </c>
-      <c r="D64" s="10" t="inlineStr">
+      <c r="D64" s="12" t="inlineStr">
         <is>
           <t>Daftar lengkap siap belanja untuk 1 unit</t>
         </is>
@@ -4147,7 +4179,7 @@
       </c>
       <c r="F64" s="16" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G64" s="16" t="inlineStr">
@@ -4165,7 +4197,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J64" s="10" t="inlineStr">
+      <c r="J64" s="12" t="inlineStr">
         <is>
           <t>sheet Komponen</t>
         </is>
@@ -4177,17 +4209,17 @@
           <t>7.2</t>
         </is>
       </c>
-      <c r="B65" s="10" t="inlineStr">
+      <c r="B65" s="12" t="inlineStr">
         <is>
           <t>Fase 7 - Duplikasi &amp; Produksi</t>
         </is>
       </c>
-      <c r="C65" s="10" t="inlineStr">
+      <c r="C65" s="12" t="inlineStr">
         <is>
           <t>Tulis panduan rakit ulang langkah demi langkah</t>
         </is>
       </c>
-      <c r="D65" s="10" t="inlineStr">
+      <c r="D65" s="12" t="inlineStr">
         <is>
           <t>Orang lain bisa mengikuti tanpa bertanya</t>
         </is>
@@ -4197,7 +4229,7 @@
       </c>
       <c r="F65" s="16" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G65" s="16" t="inlineStr">
@@ -4215,7 +4247,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J65" s="10" t="inlineStr">
+      <c r="J65" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4227,17 +4259,17 @@
           <t>7.3</t>
         </is>
       </c>
-      <c r="B66" s="10" t="inlineStr">
+      <c r="B66" s="12" t="inlineStr">
         <is>
           <t>Fase 7 - Duplikasi &amp; Produksi</t>
         </is>
       </c>
-      <c r="C66" s="10" t="inlineStr">
+      <c r="C66" s="12" t="inlineStr">
         <is>
           <t>Standarkan IP per unit (unit 2: .51 dan .61)</t>
         </is>
       </c>
-      <c r="D66" s="10" t="inlineStr">
+      <c r="D66" s="12" t="inlineStr">
         <is>
           <t>Dua mobil bisa menyala bersamaan tanpa bentrok</t>
         </is>
@@ -4247,7 +4279,7 @@
       </c>
       <c r="F66" s="16" t="inlineStr">
         <is>
-          <t>D9</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G66" s="16" t="inlineStr">
@@ -4265,7 +4297,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J66" s="10" t="inlineStr">
+      <c r="J66" s="12" t="inlineStr">
         <is>
           <t>config.h</t>
         </is>
@@ -4277,17 +4309,17 @@
           <t>7.4</t>
         </is>
       </c>
-      <c r="B67" s="10" t="inlineStr">
+      <c r="B67" s="12" t="inlineStr">
         <is>
           <t>Fase 7 - Duplikasi &amp; Produksi</t>
         </is>
       </c>
-      <c r="C67" s="10" t="inlineStr">
+      <c r="C67" s="12" t="inlineStr">
         <is>
           <t>Buat opsi SSID/IP per unit di config</t>
         </is>
       </c>
-      <c r="D67" s="10" t="inlineStr">
+      <c r="D67" s="12" t="inlineStr">
         <is>
           <t>Tidak perlu mengedit kode tiap merakit unit baru</t>
         </is>
@@ -4297,7 +4329,7 @@
       </c>
       <c r="F67" s="16" t="inlineStr">
         <is>
-          <t>D9</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G67" s="16" t="inlineStr">
@@ -4315,7 +4347,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J67" s="10" t="inlineStr">
+      <c r="J67" s="12" t="inlineStr">
         <is>
           <t>config.h</t>
         </is>
@@ -4347,7 +4379,7 @@
       </c>
       <c r="F68" s="17" t="inlineStr">
         <is>
-          <t>D9</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G68" s="17" t="inlineStr">
@@ -4377,17 +4409,17 @@
           <t>7.6</t>
         </is>
       </c>
-      <c r="B69" s="10" t="inlineStr">
+      <c r="B69" s="12" t="inlineStr">
         <is>
           <t>Fase 7 - Duplikasi &amp; Produksi</t>
         </is>
       </c>
-      <c r="C69" s="10" t="inlineStr">
+      <c r="C69" s="12" t="inlineStr">
         <is>
           <t>Catat semua kendala saat merakit unit ke-2</t>
         </is>
       </c>
-      <c r="D69" s="10" t="inlineStr">
+      <c r="D69" s="12" t="inlineStr">
         <is>
           <t>Daftar revisi konkret untuk panduan</t>
         </is>
@@ -4397,7 +4429,7 @@
       </c>
       <c r="F69" s="16" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G69" s="16" t="inlineStr">
@@ -4415,7 +4447,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J69" s="10" t="inlineStr">
+      <c r="J69" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4427,17 +4459,17 @@
           <t>7.7</t>
         </is>
       </c>
-      <c r="B70" s="10" t="inlineStr">
+      <c r="B70" s="12" t="inlineStr">
         <is>
           <t>Fase 7 - Duplikasi &amp; Produksi</t>
         </is>
       </c>
-      <c r="C70" s="10" t="inlineStr">
+      <c r="C70" s="12" t="inlineStr">
         <is>
           <t>Revisi panduan berdasarkan temuan unit ke-2</t>
         </is>
       </c>
-      <c r="D70" s="10" t="inlineStr">
+      <c r="D70" s="12" t="inlineStr">
         <is>
           <t>Panduan versi 2 yang sudah teruji</t>
         </is>
@@ -4447,7 +4479,7 @@
       </c>
       <c r="F70" s="16" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G70" s="16" t="inlineStr">
@@ -4465,7 +4497,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J70" s="10" t="inlineStr">
+      <c r="J70" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4477,17 +4509,17 @@
           <t>7.8</t>
         </is>
       </c>
-      <c r="B71" s="10" t="inlineStr">
+      <c r="B71" s="12" t="inlineStr">
         <is>
           <t>Fase 7 - Duplikasi &amp; Produksi</t>
         </is>
       </c>
-      <c r="C71" s="10" t="inlineStr">
+      <c r="C71" s="12" t="inlineStr">
         <is>
           <t>Evaluasi ganti L298N -&gt; BTS7960</t>
         </is>
       </c>
-      <c r="D71" s="10" t="inlineStr">
+      <c r="D71" s="12" t="inlineStr">
         <is>
           <t>L298N buang 2-2,5 V dan tanpa proteksi arus</t>
         </is>
@@ -4497,7 +4529,7 @@
       </c>
       <c r="F71" s="16" t="inlineStr">
         <is>
-          <t>D11</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G71" s="16" t="inlineStr">
@@ -4515,7 +4547,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J71" s="10" t="inlineStr">
+      <c r="J71" s="12" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
@@ -4527,17 +4559,17 @@
           <t>7.9</t>
         </is>
       </c>
-      <c r="B72" s="10" t="inlineStr">
+      <c r="B72" s="12" t="inlineStr">
         <is>
           <t>Fase 7 - Duplikasi &amp; Produksi</t>
         </is>
       </c>
-      <c r="C72" s="10" t="inlineStr">
+      <c r="C72" s="12" t="inlineStr">
         <is>
           <t>Evaluasi PCB custom pengganti kabel jumper</t>
         </is>
       </c>
-      <c r="D72" s="10" t="inlineStr">
+      <c r="D72" s="12" t="inlineStr">
         <is>
           <t>Keandalan naik, waktu rakit turun drastis</t>
         </is>
@@ -4547,7 +4579,7 @@
       </c>
       <c r="F72" s="16" t="inlineStr">
         <is>
-          <t>D11</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G72" s="16" t="inlineStr">
@@ -4565,7 +4597,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J72" s="10" t="inlineStr">
+      <c r="J72" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4577,17 +4609,17 @@
           <t>7.10</t>
         </is>
       </c>
-      <c r="B73" s="10" t="inlineStr">
+      <c r="B73" s="12" t="inlineStr">
         <is>
           <t>Fase 7 - Duplikasi &amp; Produksi</t>
         </is>
       </c>
-      <c r="C73" s="10" t="inlineStr">
+      <c r="C73" s="12" t="inlineStr">
         <is>
           <t>Evaluasi baterai lebih besar</t>
         </is>
       </c>
-      <c r="D73" s="10" t="inlineStr">
+      <c r="D73" s="12" t="inlineStr">
         <is>
           <t>Target runtime &gt; 15 menit (sekarang 5-8 menit)</t>
         </is>
@@ -4597,7 +4629,7 @@
       </c>
       <c r="F73" s="16" t="inlineStr">
         <is>
-          <t>D11</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G73" s="16" t="inlineStr">
@@ -4615,7 +4647,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J73" s="10" t="inlineStr">
+      <c r="J73" s="12" t="inlineStr">
         <is>
           <t>wiring 2</t>
         </is>
@@ -4627,17 +4659,17 @@
           <t>7.11</t>
         </is>
       </c>
-      <c r="B74" s="10" t="inlineStr">
+      <c r="B74" s="12" t="inlineStr">
         <is>
           <t>Fase 7 - Duplikasi &amp; Produksi</t>
         </is>
       </c>
-      <c r="C74" s="10" t="inlineStr">
+      <c r="C74" s="12" t="inlineStr">
         <is>
           <t>Buat template config per unit</t>
         </is>
       </c>
-      <c r="D74" s="10" t="inlineStr">
+      <c r="D74" s="12" t="inlineStr">
         <is>
           <t>unit-1.yaml, unit-2.yaml siap pakai</t>
         </is>
@@ -4647,7 +4679,7 @@
       </c>
       <c r="F74" s="16" t="inlineStr">
         <is>
-          <t>D11</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G74" s="16" t="inlineStr">
@@ -4665,7 +4697,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="J74" s="10" t="inlineStr">
+      <c r="J74" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4710,23 +4742,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="7" customWidth="1" min="12" max="12"/>
-    <col width="7" customWidth="1" min="13" max="13"/>
-    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4736,15 +4761,16 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
+    <row r="2" ht="74" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Angka = total jam tugas fase itu yang dijadwalkan di hari tersebut. D0 = pekerjaan yang sudah selesai. Hari bersifat relatif, bukan tanggal.</t>
+          <t>Angka = total jam tugas fase itu yang dijadwalkan di hari tersebut. Hari bersifat relatif, bukan tanggal. D0 = pekerjaan yang sudah selesai.
+TARGET 3 HARI mencakup Fase 1-5, yaitu jalur menuju mobil yang berfungsi dan teruji (21,4 jam, sekitar 7 jam per hari). Fase 6 (finalisasi) dan Fase 7 (duplikasi) berjumlah 35 jam dan sengaja TIDAK dipaksa masuk ke 3 hari itu - memadatkan semuanya berarti sekitar 19 jam per hari. Keduanya ditandai 'Lanjutan' karena memang pekerjaan setelah unit pertama terbukti jalan.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
@@ -4771,52 +4797,17 @@
       </c>
       <c r="F4" s="22" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>Lanjutan</t>
         </is>
       </c>
       <c r="G4" s="22" t="inlineStr">
         <is>
-          <t>D5</t>
-        </is>
-      </c>
-      <c r="H4" s="22" t="inlineStr">
-        <is>
-          <t>D6</t>
-        </is>
-      </c>
-      <c r="I4" s="22" t="inlineStr">
-        <is>
-          <t>D7</t>
-        </is>
-      </c>
-      <c r="J4" s="22" t="inlineStr">
-        <is>
-          <t>D8</t>
-        </is>
-      </c>
-      <c r="K4" s="22" t="inlineStr">
-        <is>
-          <t>D9</t>
-        </is>
-      </c>
-      <c r="L4" s="22" t="inlineStr">
-        <is>
-          <t>D10</t>
-        </is>
-      </c>
-      <c r="M4" s="22" t="inlineStr">
-        <is>
-          <t>D11</t>
-        </is>
-      </c>
-      <c r="N4" s="22" t="inlineStr">
-        <is>
           <t>Total</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Fase 0 - Verifikasi Meja</t>
         </is>
@@ -4841,41 +4832,13 @@
         <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A5,ToDo!$F$5:$F$74,F$4)</f>
         <v/>
       </c>
-      <c r="G5" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A5,ToDo!$F$5:$F$74,G$4)</f>
-        <v/>
-      </c>
-      <c r="H5" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A5,ToDo!$F$5:$F$74,H$4)</f>
-        <v/>
-      </c>
-      <c r="I5" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A5,ToDo!$F$5:$F$74,I$4)</f>
-        <v/>
-      </c>
-      <c r="J5" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A5,ToDo!$F$5:$F$74,J$4)</f>
-        <v/>
-      </c>
-      <c r="K5" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A5,ToDo!$F$5:$F$74,K$4)</f>
-        <v/>
-      </c>
-      <c r="L5" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A5,ToDo!$F$5:$F$74,L$4)</f>
-        <v/>
-      </c>
-      <c r="M5" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A5,ToDo!$F$5:$F$74,M$4)</f>
-        <v/>
-      </c>
-      <c r="N5" s="21">
-        <f>SUM(B5:M5)</f>
+      <c r="G5" s="21">
+        <f>SUM(B5:F5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Fase 1 - Wiring &amp; Daya</t>
         </is>
@@ -4900,41 +4863,13 @@
         <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A6,ToDo!$F$5:$F$74,F$4)</f>
         <v/>
       </c>
-      <c r="G6" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A6,ToDo!$F$5:$F$74,G$4)</f>
-        <v/>
-      </c>
-      <c r="H6" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A6,ToDo!$F$5:$F$74,H$4)</f>
-        <v/>
-      </c>
-      <c r="I6" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A6,ToDo!$F$5:$F$74,I$4)</f>
-        <v/>
-      </c>
-      <c r="J6" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A6,ToDo!$F$5:$F$74,J$4)</f>
-        <v/>
-      </c>
-      <c r="K6" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A6,ToDo!$F$5:$F$74,K$4)</f>
-        <v/>
-      </c>
-      <c r="L6" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A6,ToDo!$F$5:$F$74,L$4)</f>
-        <v/>
-      </c>
-      <c r="M6" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A6,ToDo!$F$5:$F$74,M$4)</f>
-        <v/>
-      </c>
-      <c r="N6" s="21">
-        <f>SUM(B6:M6)</f>
+      <c r="G6" s="21">
+        <f>SUM(B6:F6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Fase 2 - Flash &amp; Bench</t>
         </is>
@@ -4959,41 +4894,13 @@
         <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A7,ToDo!$F$5:$F$74,F$4)</f>
         <v/>
       </c>
-      <c r="G7" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A7,ToDo!$F$5:$F$74,G$4)</f>
-        <v/>
-      </c>
-      <c r="H7" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A7,ToDo!$F$5:$F$74,H$4)</f>
-        <v/>
-      </c>
-      <c r="I7" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A7,ToDo!$F$5:$F$74,I$4)</f>
-        <v/>
-      </c>
-      <c r="J7" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A7,ToDo!$F$5:$F$74,J$4)</f>
-        <v/>
-      </c>
-      <c r="K7" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A7,ToDo!$F$5:$F$74,K$4)</f>
-        <v/>
-      </c>
-      <c r="L7" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A7,ToDo!$F$5:$F$74,L$4)</f>
-        <v/>
-      </c>
-      <c r="M7" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A7,ToDo!$F$5:$F$74,M$4)</f>
-        <v/>
-      </c>
-      <c r="N7" s="21">
-        <f>SUM(B7:M7)</f>
+      <c r="G7" s="21">
+        <f>SUM(B7:F7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Fase 3 - Failsafe &amp; Integrasi</t>
         </is>
@@ -5018,41 +4925,13 @@
         <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A8,ToDo!$F$5:$F$74,F$4)</f>
         <v/>
       </c>
-      <c r="G8" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A8,ToDo!$F$5:$F$74,G$4)</f>
-        <v/>
-      </c>
-      <c r="H8" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A8,ToDo!$F$5:$F$74,H$4)</f>
-        <v/>
-      </c>
-      <c r="I8" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A8,ToDo!$F$5:$F$74,I$4)</f>
-        <v/>
-      </c>
-      <c r="J8" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A8,ToDo!$F$5:$F$74,J$4)</f>
-        <v/>
-      </c>
-      <c r="K8" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A8,ToDo!$F$5:$F$74,K$4)</f>
-        <v/>
-      </c>
-      <c r="L8" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A8,ToDo!$F$5:$F$74,L$4)</f>
-        <v/>
-      </c>
-      <c r="M8" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A8,ToDo!$F$5:$F$74,M$4)</f>
-        <v/>
-      </c>
-      <c r="N8" s="21">
-        <f>SUM(B8:M8)</f>
+      <c r="G8" s="21">
+        <f>SUM(B8:F8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Fase 4 - Uji Lantai &amp; Tuning</t>
         </is>
@@ -5077,41 +4956,13 @@
         <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A9,ToDo!$F$5:$F$74,F$4)</f>
         <v/>
       </c>
-      <c r="G9" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A9,ToDo!$F$5:$F$74,G$4)</f>
-        <v/>
-      </c>
-      <c r="H9" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A9,ToDo!$F$5:$F$74,H$4)</f>
-        <v/>
-      </c>
-      <c r="I9" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A9,ToDo!$F$5:$F$74,I$4)</f>
-        <v/>
-      </c>
-      <c r="J9" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A9,ToDo!$F$5:$F$74,J$4)</f>
-        <v/>
-      </c>
-      <c r="K9" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A9,ToDo!$F$5:$F$74,K$4)</f>
-        <v/>
-      </c>
-      <c r="L9" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A9,ToDo!$F$5:$F$74,L$4)</f>
-        <v/>
-      </c>
-      <c r="M9" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A9,ToDo!$F$5:$F$74,M$4)</f>
-        <v/>
-      </c>
-      <c r="N9" s="21">
-        <f>SUM(B9:M9)</f>
+      <c r="G9" s="21">
+        <f>SUM(B9:F9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Fase 5 - Pindah ke LattePanda</t>
         </is>
@@ -5136,41 +4987,13 @@
         <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A10,ToDo!$F$5:$F$74,F$4)</f>
         <v/>
       </c>
-      <c r="G10" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A10,ToDo!$F$5:$F$74,G$4)</f>
-        <v/>
-      </c>
-      <c r="H10" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A10,ToDo!$F$5:$F$74,H$4)</f>
-        <v/>
-      </c>
-      <c r="I10" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A10,ToDo!$F$5:$F$74,I$4)</f>
-        <v/>
-      </c>
-      <c r="J10" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A10,ToDo!$F$5:$F$74,J$4)</f>
-        <v/>
-      </c>
-      <c r="K10" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A10,ToDo!$F$5:$F$74,K$4)</f>
-        <v/>
-      </c>
-      <c r="L10" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A10,ToDo!$F$5:$F$74,L$4)</f>
-        <v/>
-      </c>
-      <c r="M10" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A10,ToDo!$F$5:$F$74,M$4)</f>
-        <v/>
-      </c>
-      <c r="N10" s="21">
-        <f>SUM(B10:M10)</f>
+      <c r="G10" s="21">
+        <f>SUM(B10:F10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Fase 6 - Finalisasi</t>
         </is>
@@ -5195,41 +5018,13 @@
         <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A11,ToDo!$F$5:$F$74,F$4)</f>
         <v/>
       </c>
-      <c r="G11" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A11,ToDo!$F$5:$F$74,G$4)</f>
-        <v/>
-      </c>
-      <c r="H11" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A11,ToDo!$F$5:$F$74,H$4)</f>
-        <v/>
-      </c>
-      <c r="I11" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A11,ToDo!$F$5:$F$74,I$4)</f>
-        <v/>
-      </c>
-      <c r="J11" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A11,ToDo!$F$5:$F$74,J$4)</f>
-        <v/>
-      </c>
-      <c r="K11" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A11,ToDo!$F$5:$F$74,K$4)</f>
-        <v/>
-      </c>
-      <c r="L11" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A11,ToDo!$F$5:$F$74,L$4)</f>
-        <v/>
-      </c>
-      <c r="M11" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A11,ToDo!$F$5:$F$74,M$4)</f>
-        <v/>
-      </c>
-      <c r="N11" s="21">
-        <f>SUM(B11:M11)</f>
+      <c r="G11" s="21">
+        <f>SUM(B11:F11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Fase 7 - Duplikasi &amp; Produksi</t>
         </is>
@@ -5254,41 +5049,13 @@
         <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A12,ToDo!$F$5:$F$74,F$4)</f>
         <v/>
       </c>
-      <c r="G12" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A12,ToDo!$F$5:$F$74,G$4)</f>
-        <v/>
-      </c>
-      <c r="H12" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A12,ToDo!$F$5:$F$74,H$4)</f>
-        <v/>
-      </c>
-      <c r="I12" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A12,ToDo!$F$5:$F$74,I$4)</f>
-        <v/>
-      </c>
-      <c r="J12" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A12,ToDo!$F$5:$F$74,J$4)</f>
-        <v/>
-      </c>
-      <c r="K12" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A12,ToDo!$F$5:$F$74,K$4)</f>
-        <v/>
-      </c>
-      <c r="L12" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A12,ToDo!$F$5:$F$74,L$4)</f>
-        <v/>
-      </c>
-      <c r="M12" s="23">
-        <f>SUMIFS(ToDo!$E$5:$E$74,ToDo!$B$5:$B$74,$A12,ToDo!$F$5:$F$74,M$4)</f>
-        <v/>
-      </c>
-      <c r="N12" s="21">
-        <f>SUM(B12:M12)</f>
+      <c r="G12" s="21">
+        <f>SUM(B12:F12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>TOTAL / HARI</t>
         </is>
@@ -5317,40 +5084,12 @@
         <f>SUM(G5:G12)</f>
         <v/>
       </c>
-      <c r="H13" s="24">
-        <f>SUM(H5:H12)</f>
-        <v/>
-      </c>
-      <c r="I13" s="24">
-        <f>SUM(I5:I12)</f>
-        <v/>
-      </c>
-      <c r="J13" s="24">
-        <f>SUM(J5:J12)</f>
-        <v/>
-      </c>
-      <c r="K13" s="24">
-        <f>SUM(K5:K12)</f>
-        <v/>
-      </c>
-      <c r="L13" s="24">
-        <f>SUM(L5:L12)</f>
-        <v/>
-      </c>
-      <c r="M13" s="24">
-        <f>SUM(M5:M12)</f>
-        <v/>
-      </c>
-      <c r="N13" s="24">
-        <f>SUM(N5:N12)</f>
-        <v/>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:M12">
+  <conditionalFormatting sqref="B5:F12">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -5392,49 +5131,49 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Komponen</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Spesifikasi</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>Jumlah</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>Harga Satuan (Rp)</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr">
         <is>
           <t>Subtotal (Rp)</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>Catatan</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>LattePanda</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Ground station</t>
         </is>
@@ -5452,19 +5191,19 @@
         <f>IFERROR(C5*E5,0)</f>
         <v/>
       </c>
-      <c r="G5" s="10" t="inlineStr">
+      <c r="G5" s="12" t="inlineStr">
         <is>
           <t>Tempat stir PXN dicolok</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Stir PXN V9 (V9GEN2) + pedal</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>H-pattern shifter 6 gigi + R</t>
         </is>
@@ -5482,19 +5221,19 @@
         <f>IFERROR(C6*E6,0)</f>
         <v/>
       </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="G6" s="12" t="inlineStr">
         <is>
           <t>Sudah dikalibrasi</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>ESP32 Dev Module</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>38 pin</t>
         </is>
@@ -5512,19 +5251,19 @@
         <f>IFERROR(C7*E7,0)</f>
         <v/>
       </c>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="G7" s="12" t="inlineStr">
         <is>
           <t>Otak mobil</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Seeed XIAO ESP32S3 Sense</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>dengan papan kamera + antena u.FL</t>
         </is>
@@ -5542,19 +5281,19 @@
         <f>IFERROR(C8*E8,0)</f>
         <v/>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="G8" s="12" t="inlineStr">
         <is>
           <t>Kamera FPV</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>L298N</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>modul driver motor</t>
         </is>
@@ -5572,19 +5311,19 @@
         <f>IFERROR(C9*E9,0)</f>
         <v/>
       </c>
-      <c r="G9" s="10" t="inlineStr">
+      <c r="G9" s="12" t="inlineStr">
         <is>
           <t>Lepas jumper ENA dan 5V</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Servo digital 25g</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>stall ~1-1,5 A</t>
         </is>
@@ -5602,19 +5341,19 @@
         <f>IFERROR(C10*E10,0)</f>
         <v/>
       </c>
-      <c r="G10" s="10" t="inlineStr">
+      <c r="G10" s="12" t="inlineStr">
         <is>
           <t>Kemudi, sinyal ke GPIO 13</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Motor DC belakang</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>12 V</t>
         </is>
@@ -5632,19 +5371,19 @@
         <f>IFERROR(C11*E11,0)</f>
         <v/>
       </c>
-      <c r="G11" s="10" t="inlineStr">
+      <c r="G11" s="12" t="inlineStr">
         <is>
           <t>Lewat OUT1/OUT2</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>LiPo 4S 850 mAh</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>14,8 V nominal</t>
         </is>
@@ -5662,19 +5401,19 @@
         <f>IFERROR(C12*E12,0)</f>
         <v/>
       </c>
-      <c r="G12" s="10" t="inlineStr">
+      <c r="G12" s="12" t="inlineStr">
         <is>
           <t>Runtime 5-8 menit</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Step-down #1</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>4S -&gt; 12 V, &gt;= 3 A (XL4015/LM2596)</t>
         </is>
@@ -5692,19 +5431,19 @@
         <f>IFERROR(C13*E13,0)</f>
         <v/>
       </c>
-      <c r="G13" s="10" t="inlineStr">
+      <c r="G13" s="12" t="inlineStr">
         <is>
           <t>Catu motor</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Step-down #2</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>4S -&gt; 5 V, &gt;= 3 A</t>
         </is>
@@ -5722,19 +5461,19 @@
         <f>IFERROR(C14*E14,0)</f>
         <v/>
       </c>
-      <c r="G14" s="10" t="inlineStr">
+      <c r="G14" s="12" t="inlineStr">
         <is>
           <t>Servo + kedua ESP32</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>Elko 1000uF / 25V</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>low-ESR</t>
         </is>
@@ -5752,19 +5491,19 @@
         <f>IFERROR(C15*E15,0)</f>
         <v/>
       </c>
-      <c r="G15" s="10" t="inlineStr">
+      <c r="G15" s="12" t="inlineStr">
         <is>
           <t>Di jalur 5V servo - WAJIB</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Elko 470uF / 16V</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>low-ESR</t>
         </is>
@@ -5782,19 +5521,19 @@
         <f>IFERROR(C16*E16,0)</f>
         <v/>
       </c>
-      <c r="G16" s="10" t="inlineStr">
+      <c r="G16" s="12" t="inlineStr">
         <is>
           <t>Di 5V kamera - WAJIB</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>Elko 470uF / 25V</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>low-ESR</t>
         </is>
@@ -5812,19 +5551,19 @@
         <f>IFERROR(C17*E17,0)</f>
         <v/>
       </c>
-      <c r="G17" s="10" t="inlineStr">
+      <c r="G17" s="12" t="inlineStr">
         <is>
           <t>Di Vs L298N</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>Kapasitor keramik 100nF</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5842,19 +5581,19 @@
         <f>IFERROR(C18*E18,0)</f>
         <v/>
       </c>
-      <c r="G18" s="10" t="inlineStr">
+      <c r="G18" s="12" t="inlineStr">
         <is>
           <t>3 di motor, sisanya bypass</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Resistor 100k</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>1% kalau ada</t>
         </is>
@@ -5872,19 +5611,19 @@
         <f>IFERROR(C19*E19,0)</f>
         <v/>
       </c>
-      <c r="G19" s="10" t="inlineStr">
+      <c r="G19" s="12" t="inlineStr">
         <is>
           <t>Pembagi tegangan baterai</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>Resistor 22k</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>1% kalau ada</t>
         </is>
@@ -5902,19 +5641,19 @@
         <f>IFERROR(C20*E20,0)</f>
         <v/>
       </c>
-      <c r="G20" s="10" t="inlineStr">
+      <c r="G20" s="12" t="inlineStr">
         <is>
           <t>Pembagi tegangan baterai</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>Resistor 10k</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5932,19 +5671,19 @@
         <f>IFERROR(C21*E21,0)</f>
         <v/>
       </c>
-      <c r="G21" s="10" t="inlineStr">
+      <c r="G21" s="12" t="inlineStr">
         <is>
           <t>Pulldown ENA / IN1 / IN2</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>Alarm LiPo 4S</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>buzzer per-sel</t>
         </is>
@@ -5962,19 +5701,19 @@
         <f>IFERROR(C22*E22,0)</f>
         <v/>
       </c>
-      <c r="G22" s="10" t="inlineStr">
+      <c r="G22" s="12" t="inlineStr">
         <is>
           <t>Peringatan tegangan mandiri</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>Kabel USB-C</t>
         </is>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>data, bukan charge-only</t>
         </is>
@@ -5992,19 +5731,19 @@
         <f>IFERROR(C23*E23,0)</f>
         <v/>
       </c>
-      <c r="G23" s="10" t="inlineStr">
+      <c r="G23" s="12" t="inlineStr">
         <is>
           <t>Flash XIAO</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>Kabel jumper + heat shrink</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6022,7 +5761,7 @@
         <f>IFERROR(C24*E24,0)</f>
         <v/>
       </c>
-      <c r="G24" s="10" t="inlineStr">
+      <c r="G24" s="12" t="inlineStr">
         <is>
           <t>Perakitan</t>
         </is>
@@ -6079,39 +5818,39 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Risiko</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Kemungkinan</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>Dampak</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>Penyebab</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>Mitigasi</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr">
         <is>
           <t>Tugas Terkait</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Kamera reboot saat servo bergerak</t>
         </is>
@@ -6126,12 +5865,12 @@
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Rel 5V drop saat servo menyentak</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>Elko 1000uF di servo + 470uF di kamera. Kalau tetap: step-down ketiga khusus ESP32</t>
         </is>
@@ -6143,7 +5882,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Motor hanya mati / kencang penuh</t>
         </is>
@@ -6158,12 +5897,12 @@
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Jumper ENA belum dilepas</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
         <is>
           <t>Lepas jumper ENA di L298N</t>
         </is>
@@ -6175,7 +5914,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Servo tidak bergerak sama sekali</t>
         </is>
@@ -6190,12 +5929,12 @@
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Sinyal masih di GPIO 34 yang input-only</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Pindahkan kabel sinyal ke GPIO 13</t>
         </is>
@@ -6207,7 +5946,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Kamera gagal init di XIAO</t>
         </is>
@@ -6222,12 +5961,12 @@
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>PSRAM masih Disabled, atau papan Sense kurang rapat</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>Set PSRAM = OPI PSRAM; tekan papan Sense sampai bunyi klik</t>
         </is>
@@ -6239,7 +5978,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Mobil tidak ditemukan ground station</t>
         </is>
@@ -6254,12 +5993,12 @@
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Subnet hotspot bukan 192.168.137.x</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Cek IP di Serial Monitor, sesuaikan config.h dan config.yaml</t>
         </is>
@@ -6271,7 +6010,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Motor tidak berhenti saat sinyal putus</t>
         </is>
@@ -6286,12 +6025,12 @@
           <t>Sangat tinggi</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Failsafe gagal - mobil bisa lari tak terkendali</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>Uji 3.1 WAJIB lolos sebelum turun ke lantai</t>
         </is>
@@ -6303,7 +6042,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Perilaku acak, servo bergetar sendiri</t>
         </is>
@@ -6318,12 +6057,12 @@
           <t>Sedang</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Ground tidak menyatu di satu titik</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>Star ground semua modul dekat terminal negatif baterai</t>
         </is>
@@ -6335,7 +6074,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Video penuh garis / WiFi drop</t>
         </is>
@@ -6350,12 +6089,12 @@
           <t>Sedang</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Noise percikan sikat motor</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="E12" s="12" t="inlineStr">
         <is>
           <t>3 keramik 100nF di badan motor; jauhkan kabel motor dari kamera</t>
         </is>
@@ -6367,7 +6106,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Ping melonjak acak ratusan ms</t>
         </is>
@@ -6382,12 +6121,12 @@
           <t>Sedang</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>WiFi power save aktif</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="E13" s="12" t="inlineStr">
         <is>
           <t>Pastikan WiFi.setSleep(false) ada di kedua firmware</t>
         </is>
@@ -6399,7 +6138,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Tegangan HUD tidak cocok multimeter</t>
         </is>
@@ -6414,12 +6153,12 @@
           <t>Rendah</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>Toleransi resistor 5% - bisa meleset 0,8 V di 4S</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="E14" s="12" t="inlineStr">
         <is>
           <t>Kalibrasi VBAT_DIVIDER_RATIO</t>
         </is>
@@ -6431,7 +6170,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>Runtime terlalu pendek</t>
         </is>
@@ -6446,12 +6185,12 @@
           <t>Sedang</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>4S 850 mAh memang kecil</t>
         </is>
       </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr">
         <is>
           <t>Batas kapasitas, bukan software. Perlu paket lebih besar</t>
         </is>
@@ -6463,7 +6202,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>L298N kepanasan</t>
         </is>
@@ -6478,12 +6217,12 @@
           <t>Sedang</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>Buang 2-2,5 V, tanpa proteksi arus</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="E16" s="12" t="inlineStr">
         <is>
           <t>Cek suhu tiap uji. Untuk produksi pertimbangkan BTS7960</t>
         </is>
@@ -6495,7 +6234,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>Servo rusak karena menahan di ujung</t>
         </is>
@@ -6510,12 +6249,12 @@
           <t>Sedang</t>
         </is>
       </c>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>SERVO_MIN/MAX_US terlalu lebar</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>Setel bertahap 50us, berhenti begitu mendengung</t>
         </is>
@@ -6527,7 +6266,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>Enumerasi USB beda di LattePanda</t>
         </is>
@@ -6542,12 +6281,12 @@
           <t>Rendah</t>
         </is>
       </c>
-      <c r="D18" s="10" t="inlineStr">
+      <c r="D18" s="12" t="inlineStr">
         <is>
           <t>Indeks joystick berubah antar mesin</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="E18" s="12" t="inlineStr">
         <is>
           <t>Jalankan calibrate.py ulang di LattePanda</t>
         </is>

</xml_diff>